<commit_message>
Daily EOD data and reports for 2026-10-20
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20261020.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20261020.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.71</v>
+        <v>1.695</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.05</v>
+        <v>-0.065</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-2.84%</t>
+          <t>-3.69%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>261939.51</v>
+        <v>259641.8</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-7659.05</v>
+        <v>-9956.76</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.425</v>
+        <v>2.405</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.045</v>
+        <v>-0.065</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.82%</t>
+          <t>-2.63%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>169750</v>
+        <v>168350</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-3150</v>
+        <v>-4550</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>59.14</v>
+        <v>59.39</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-1.32</v>
+        <v>-1.07</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-2.18%</t>
+          <t>-1.77%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>473120</v>
+        <v>475120</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-10560</v>
+        <v>-8560</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0</v>
+        <v>0.006</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.004</v>
+        <v>0.002</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0</v>
+        <v>264.54</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-176.36</v>
+        <v>88.18000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>153.16</v>
+        <v>154.89</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-2.23</v>
+        <v>-0.5</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-1.44%</t>
+          <t>-0.32%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.005</v>
+        <v>0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.61%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>8150</v>
+        <v>8200</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>194.595</v>
+        <v>196.68</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.545</v>
+        <v>2.63</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>1.36%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>778380</v>
+        <v>786720</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>2180</v>
+        <v>10520</v>
       </c>
     </row>
     <row r="11">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>11.76</v>
+        <v>11.56</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.21</v>
+        <v>-0.41</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-1.75%</t>
+          <t>-3.43%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>35809.2</v>
+        <v>35200.2</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-639.45</v>
+        <v>-1248.45</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0</v>
+        <v>0.081</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.08</v>
+        <v>0.001</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>1.25%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0</v>
+        <v>762.37</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-752.96</v>
+        <v>9.41</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.08500000000000001</v>
+        <v>0.002</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>2.35%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>522</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-510</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.87</v>
+        <v>35.07</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.54</v>
+        <v>-0.34</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-1.52%</t>
+          <t>-0.96%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>33.695</v>
+        <v>33.71</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.335</v>
+        <v>-0.32</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-0.98%</t>
+          <t>-0.94%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>43399.16</v>
+        <v>43418.48</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-431.48</v>
+        <v>-412.16</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1774847.87</v>
+        <v>1782499.39</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-23349.3</v>
+        <v>-15697.78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>